<commit_message>
added 2 new feature: 1. step-level validation for some data, 2. PDF download verification.
</commit_message>
<xml_diff>
--- a/Test_DemoWebShop/TestData/TestData.xlsx
+++ b/Test_DemoWebShop/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riseup\Katalon Studio\Test_Demo\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C7BB20-E3B6-4597-890B-D5D464A7228C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA31C1B-4B82-4C4D-A8D8-354637F7D9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>itemsWithQuantity</t>
   </si>
@@ -39,20 +39,32 @@
     <t>Blue Jeans:2,Blue and green Sneaker:3,Casual Golf Belt:4</t>
   </si>
   <si>
-    <t>3rd Album:4,Black &amp; White Diamond Heart:2</t>
+    <t>countryCode</t>
+  </si>
+  <si>
+    <t>zipCode</t>
+  </si>
+  <si>
+    <t>shippingMethod</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -75,8 +87,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,43 +370,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.21875" customWidth="1"/>
     <col min="2" max="2" width="50.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>1229</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
+      <c r="C3">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>5488</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>